<commit_message>
Revise after peer review: robustness checks, campaign fix, SEC recall
- Fix hand_merge: press attribution to the 2025 Salesforce wave now requires
  year 2025; a 2019 TransUnion record is a separate event (202 events, 163
  hand-coded; the original 60-event sample is reproduced unchanged)
- Add src/robustness.py: detection by root cause, bounding of the
  misconfiguration contrast, recoding sensitivity (customer-managed
  campaigns, network-only codes), SEC strict rule, SEC recall against an
  external count, sample-size calculation
- SEC comparison uses the hand codes for hand-coded VCDB events
- Collector v3 searches more Item 8.01 wordings
- Second-coder package now includes the 68 SEC incidents; kappa.py accepts it
- Paper PDF and SEC workbook updated; SPI and placement model removed from
  the submission (code kept)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T1EPgqfEcJyYq1wKYDTMD9
</commit_message>
<xml_diff>
--- a/results/sec/SEC_8K_incidents_vs_VCDB.xlsx
+++ b/results/sec/SEC_8K_incidents_vs_VCDB.xlsx
@@ -53,7 +53,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">VCDB values: results/analysis_results.json (B_hand_table, B_hand_events) and results/hand/events_hand.csv (hand_root_cause), repo schennuri/breach-evidence-gap.</t>
+          <t xml:space="preserve">VCDB values: results/analysis_results.json (B_hand_table, B_hand_events) and results/hand/events_hand.csv with the hand codes from data/hand_codes/hand_codes_all.csv, repo schennuri/breach-evidence-gap.</t>
         </r>
       </text>
     </comment>
@@ -128,7 +128,7 @@
     <t xml:space="preserve">Events after merging CDK dealers</t>
   </si>
   <si>
-    <t xml:space="preserve">Table VI — SEC events vs VCDB events (hand rule)</t>
+    <t xml:space="preserve">Table VII — SEC events vs VCDB events (hand rule)</t>
   </si>
   <si>
     <t xml:space="preserve">Measure</t>
@@ -3309,11 +3309,11 @@
         <v>56</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G15" s="8" t="n">
         <f aca="false">IF(F15=0,0,E15/F15)</f>
-        <v>0.278606965174129</v>
+        <v>0.277227722772277</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>0.35</v>
@@ -3366,17 +3366,17 @@
         <v>0.169230769230769</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G17" s="8" t="n">
         <f aca="false">IF(F17=0,0,E17/F17)</f>
-        <v>0.537313432835821</v>
+        <v>0.504950495049505</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>1.3E-007</v>
+        <v>1.3E-006</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3396,17 +3396,17 @@
         <v>0</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G18" s="8" t="n">
         <f aca="false">IF(F18=0,0,E18/F18)</f>
-        <v>0.223880597014925</v>
+        <v>0.217821782178218</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>1.5E-006</v>
+        <v>1.6E-006</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>